<commit_message>
Update Danh sách VNSH03 nhận từ X-Force.xlsx
</commit_message>
<xml_diff>
--- a/5. Other/Danh sách VNSH03 nhận từ X-Force.xlsx
+++ b/5. Other/Danh sách VNSH03 nhận từ X-Force.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VNET\5. Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752E2119-950B-44EE-864F-8A9019DE8BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A39776C-2909-4BFE-9855-7B7F2758D221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{DE03BF13-5A63-4E6D-9BDA-D95C0EEDDB32}"/>
   </bookViews>
@@ -1464,9 +1464,6 @@
     <t>ID sai</t>
   </si>
   <si>
-    <t>Victory trả về, lỗi không LED trạng thái</t>
-  </si>
-  <si>
     <t>Không chốt GPS, IPEX bị lỏng</t>
   </si>
   <si>
@@ -1510,6 +1507,9 @@
   </si>
   <si>
     <t>Thiết bị đã đổi BH 1 lần nhận lại lỗi quạt gió, có phản hồi từ HTKT đèn trạng thái thiết bị không khởi động được</t>
+  </si>
+  <si>
+    <t>Victory trả về, lỗi không LED trạng thái, gửi Thịnh Aithings xử lý 21/07/2026</t>
   </si>
 </sst>
 </file>
@@ -1602,7 +1602,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1668,6 +1668,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4074,7 +4077,7 @@
         <v>185</v>
       </c>
       <c r="E126" s="17" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F126" s="20"/>
     </row>
@@ -5084,7 +5087,7 @@
       <c r="E189" s="15"/>
       <c r="F189" s="20"/>
     </row>
-    <row r="190" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A190" s="4">
         <v>189</v>
       </c>
@@ -5098,10 +5101,10 @@
         <v>103</v>
       </c>
       <c r="E190" s="17" t="s">
-        <v>478</v>
-      </c>
-      <c r="F190" s="20" t="s">
-        <v>480</v>
+        <v>493</v>
+      </c>
+      <c r="F190" s="26" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
@@ -6222,7 +6225,7 @@
         <v>103</v>
       </c>
       <c r="E260" s="17" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="F260" s="20"/>
     </row>
@@ -6408,7 +6411,7 @@
         <v>103</v>
       </c>
       <c r="E272" s="4" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F272" s="4"/>
     </row>
@@ -9211,14 +9214,14 @@
         <v>462</v>
       </c>
       <c r="B463" s="24" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C463" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D463" s="25"/>
       <c r="E463" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F463" s="20"/>
     </row>
@@ -9227,14 +9230,14 @@
         <v>463</v>
       </c>
       <c r="B464" s="24" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C464" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D464" s="25"/>
       <c r="E464" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F464" s="20"/>
     </row>
@@ -9243,14 +9246,14 @@
         <v>464</v>
       </c>
       <c r="B465" s="24" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C465" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D465" s="25"/>
       <c r="E465" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F465" s="20"/>
     </row>
@@ -9259,14 +9262,14 @@
         <v>465</v>
       </c>
       <c r="B466" s="24" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C466" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D466" s="25"/>
       <c r="E466" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F466" s="20"/>
     </row>
@@ -9275,14 +9278,14 @@
         <v>466</v>
       </c>
       <c r="B467" s="24" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C467" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D467" s="25"/>
       <c r="E467" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F467" s="20"/>
     </row>
@@ -9291,14 +9294,14 @@
         <v>467</v>
       </c>
       <c r="B468" s="24" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C468" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D468" s="25"/>
       <c r="E468" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F468" s="20"/>
     </row>
@@ -9307,14 +9310,14 @@
         <v>468</v>
       </c>
       <c r="B469" s="24" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C469" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D469" s="25"/>
       <c r="E469" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F469" s="20"/>
     </row>
@@ -9323,14 +9326,14 @@
         <v>469</v>
       </c>
       <c r="B470" s="24" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C470" s="24" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="D470" s="25"/>
       <c r="E470" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F470" s="20"/>
     </row>
@@ -9339,14 +9342,14 @@
         <v>470</v>
       </c>
       <c r="B471" s="24" t="s">
+        <v>488</v>
+      </c>
+      <c r="C471" s="24" t="s">
         <v>489</v>
-      </c>
-      <c r="C471" s="24" t="s">
-        <v>490</v>
       </c>
       <c r="D471" s="25"/>
       <c r="E471" s="15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F471" s="20"/>
     </row>

</xml_diff>